<commit_message>
shot_table.xlsx: flywheel unit dropdown (% or us); us converted from the forward side of 1500 per Flywheel::INVERTED
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/shot_table/shot_table.xlsx
+++ b/tools/shot_table/shot_table.xlsx
@@ -864,7 +864,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
-    <col min="1" max="4" width="12" customWidth="1"/>
+    <col min="1" max="5" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -885,7 +885,12 @@
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>轉速(%)</t>
+          <t>轉速</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>轉速單位</t>
         </is>
       </c>
     </row>
@@ -902,6 +907,11 @@
       <c r="D2">
         <v>42.0</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -916,6 +926,11 @@
       <c r="D3">
         <v>43.0</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -930,6 +945,11 @@
       <c r="D4">
         <v>100.0</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -944,6 +964,11 @@
       <c r="D5">
         <v>46.0</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -958,6 +983,11 @@
       <c r="D6">
         <v>100.0</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -972,9 +1002,14 @@
       <c r="D7">
         <v>80.0</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="洞口" error="洞口要是 1–9 的整數" sqref="A2:A500">
       <formula1>1</formula1>
       <formula2>9</formula2>
@@ -987,9 +1022,11 @@
       <formula1>500</formula1>
       <formula2>2500</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="轉速" error="轉速 0–100 %" sqref="D2:D500">
-      <formula1>0</formula1>
-      <formula2>100</formula2>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="轉速" error="單位 % 時 0–100；單位 us 時 1000–2000 的整數" sqref="D2:D500">
+      <formula1>OR(AND(E2="%",D2&gt;=0,D2&lt;=100),AND(E2="us",D2&gt;=1000,D2&lt;=2000,INT(D2)=D2))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="轉速單位" error="只能選 % 或 us" sqref="E2:E500">
+      <formula1>"%,us"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -1047,7 +1084,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- 第 1 列是欄位名稱。「洞口」「距離(m)」「仰角(us)」「轉速(%)」四個必須各出現一次、名稱一字不差。</t>
+          <t>- 第 1 列是欄位名稱。「洞口」「距離(m)」「仰角(us)」「轉速」「轉速單位」五個必須各出現一次、名稱一字不差。</t>
         </is>
       </c>
     </row>
@@ -1082,61 +1119,68 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- 轉速：Falcon 指令 0–100 %，最多 1 位小數。</t>
+          <t>- 轉速單位：用下拉選單選「%」或「us」，每一列可以不同。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- 列的順序不重要；空白列會略過；同一個洞口的同一個距離不能重複。</t>
+          <t>- 轉速：單位 % 時 0–100、最多 1 位小數；單位 us 時填 Dashboard「Falcon PWM」的脈寬整數，必須在正轉那一側（目前是 1000–1500），會自動換算成 %。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- 資料請放在第 2–500 列；每個洞口最多 60 個點會畫進曲線圖。</t>
+          <t>- 列的順序不重要；空白列會略過；同一個洞口的同一個距離不能重複。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>- 資料請放在第 2–500 列；每個洞口最多 60 個點會畫進曲線圖。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>- 任何一格不符合，就不會產生檔案、也不會燒錄，畫面會指出是哪一格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>沒有資料的洞</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>- 會借用同一排中間洞的值：1、7 用 4，2、8 用 5，3、9 用 6。</t>
+          <t>沒有資料的洞</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- Mega 在兩個量測點之間用直線內插；比最近的點還近就用最近的點；比最遠的點還遠就用最遠的點。</t>
+          <t>- 會借用同一排中間洞的值：1、7 用 4，2、8 用 5，3、9 用 6。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>- Mega 在兩個量測點之間用直線內插；比最近的點還近就用最近的點；比最遠的點還遠就用最遠的點。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>- 曲線圖上的轉速曲線是 Excel 的乘冪趨勢線（y = a·x^b，從原點出發），只是用來看資料合不合理、哪個點量歪了；Mega 不是照這條曲線打。</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>「圖表資料」是隱藏的工作表，由公式自動整理給曲線圖用，不用動它。</t>
         </is>
@@ -1204,7 +1248,7 @@
         <f t="array" ref="B2">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A2),0)),NA())</f>
       </c>
       <c r="C2">
-        <f t="array" ref="C2">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A2),0)),NA())</f>
+        <f t="array" ref="C2">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A2),0)),NA())</f>
       </c>
       <c r="D2">
         <f t="array" ref="D2">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),1),NA())</f>
@@ -1213,7 +1257,7 @@
         <f t="array" ref="E2">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D2),0)),NA())</f>
       </c>
       <c r="F2">
-        <f t="array" ref="F2">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D2),0)),NA())</f>
+        <f t="array" ref="F2">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D2),0)),NA())</f>
       </c>
       <c r="G2">
         <f t="array" ref="G2">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),1),NA())</f>
@@ -1222,7 +1266,7 @@
         <f t="array" ref="H2">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G2),0)),NA())</f>
       </c>
       <c r="I2">
-        <f t="array" ref="I2">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G2),0)),NA())</f>
+        <f t="array" ref="I2">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G2),0)),NA())</f>
       </c>
     </row>
     <row r="3">
@@ -1233,7 +1277,7 @@
         <f t="array" ref="B3">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A3),0)),NA())</f>
       </c>
       <c r="C3">
-        <f t="array" ref="C3">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A3),0)),NA())</f>
+        <f t="array" ref="C3">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A3),0)),NA())</f>
       </c>
       <c r="D3">
         <f t="array" ref="D3">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),2),NA())</f>
@@ -1242,7 +1286,7 @@
         <f t="array" ref="E3">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D3),0)),NA())</f>
       </c>
       <c r="F3">
-        <f t="array" ref="F3">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D3),0)),NA())</f>
+        <f t="array" ref="F3">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D3),0)),NA())</f>
       </c>
       <c r="G3">
         <f t="array" ref="G3">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),2),NA())</f>
@@ -1251,7 +1295,7 @@
         <f t="array" ref="H3">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G3),0)),NA())</f>
       </c>
       <c r="I3">
-        <f t="array" ref="I3">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G3),0)),NA())</f>
+        <f t="array" ref="I3">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G3),0)),NA())</f>
       </c>
     </row>
     <row r="4">
@@ -1262,7 +1306,7 @@
         <f t="array" ref="B4">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A4),0)),NA())</f>
       </c>
       <c r="C4">
-        <f t="array" ref="C4">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A4),0)),NA())</f>
+        <f t="array" ref="C4">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A4),0)),NA())</f>
       </c>
       <c r="D4">
         <f t="array" ref="D4">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),3),NA())</f>
@@ -1271,7 +1315,7 @@
         <f t="array" ref="E4">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D4),0)),NA())</f>
       </c>
       <c r="F4">
-        <f t="array" ref="F4">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D4),0)),NA())</f>
+        <f t="array" ref="F4">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D4),0)),NA())</f>
       </c>
       <c r="G4">
         <f t="array" ref="G4">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),3),NA())</f>
@@ -1280,7 +1324,7 @@
         <f t="array" ref="H4">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G4),0)),NA())</f>
       </c>
       <c r="I4">
-        <f t="array" ref="I4">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G4),0)),NA())</f>
+        <f t="array" ref="I4">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G4),0)),NA())</f>
       </c>
     </row>
     <row r="5">
@@ -1291,7 +1335,7 @@
         <f t="array" ref="B5">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A5),0)),NA())</f>
       </c>
       <c r="C5">
-        <f t="array" ref="C5">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A5),0)),NA())</f>
+        <f t="array" ref="C5">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A5),0)),NA())</f>
       </c>
       <c r="D5">
         <f t="array" ref="D5">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),4),NA())</f>
@@ -1300,7 +1344,7 @@
         <f t="array" ref="E5">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D5),0)),NA())</f>
       </c>
       <c r="F5">
-        <f t="array" ref="F5">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D5),0)),NA())</f>
+        <f t="array" ref="F5">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D5),0)),NA())</f>
       </c>
       <c r="G5">
         <f t="array" ref="G5">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),4),NA())</f>
@@ -1309,7 +1353,7 @@
         <f t="array" ref="H5">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G5),0)),NA())</f>
       </c>
       <c r="I5">
-        <f t="array" ref="I5">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G5),0)),NA())</f>
+        <f t="array" ref="I5">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G5),0)),NA())</f>
       </c>
     </row>
     <row r="6">
@@ -1320,7 +1364,7 @@
         <f t="array" ref="B6">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A6),0)),NA())</f>
       </c>
       <c r="C6">
-        <f t="array" ref="C6">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A6),0)),NA())</f>
+        <f t="array" ref="C6">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A6),0)),NA())</f>
       </c>
       <c r="D6">
         <f t="array" ref="D6">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),5),NA())</f>
@@ -1329,7 +1373,7 @@
         <f t="array" ref="E6">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D6),0)),NA())</f>
       </c>
       <c r="F6">
-        <f t="array" ref="F6">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D6),0)),NA())</f>
+        <f t="array" ref="F6">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D6),0)),NA())</f>
       </c>
       <c r="G6">
         <f t="array" ref="G6">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),5),NA())</f>
@@ -1338,7 +1382,7 @@
         <f t="array" ref="H6">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G6),0)),NA())</f>
       </c>
       <c r="I6">
-        <f t="array" ref="I6">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G6),0)),NA())</f>
+        <f t="array" ref="I6">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G6),0)),NA())</f>
       </c>
     </row>
     <row r="7">
@@ -1349,7 +1393,7 @@
         <f t="array" ref="B7">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A7),0)),NA())</f>
       </c>
       <c r="C7">
-        <f t="array" ref="C7">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A7),0)),NA())</f>
+        <f t="array" ref="C7">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A7),0)),NA())</f>
       </c>
       <c r="D7">
         <f t="array" ref="D7">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),6),NA())</f>
@@ -1358,7 +1402,7 @@
         <f t="array" ref="E7">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D7),0)),NA())</f>
       </c>
       <c r="F7">
-        <f t="array" ref="F7">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D7),0)),NA())</f>
+        <f t="array" ref="F7">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D7),0)),NA())</f>
       </c>
       <c r="G7">
         <f t="array" ref="G7">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),6),NA())</f>
@@ -1367,7 +1411,7 @@
         <f t="array" ref="H7">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G7),0)),NA())</f>
       </c>
       <c r="I7">
-        <f t="array" ref="I7">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G7),0)),NA())</f>
+        <f t="array" ref="I7">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G7),0)),NA())</f>
       </c>
     </row>
     <row r="8">
@@ -1378,7 +1422,7 @@
         <f t="array" ref="B8">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A8),0)),NA())</f>
       </c>
       <c r="C8">
-        <f t="array" ref="C8">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A8),0)),NA())</f>
+        <f t="array" ref="C8">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A8),0)),NA())</f>
       </c>
       <c r="D8">
         <f t="array" ref="D8">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),7),NA())</f>
@@ -1387,7 +1431,7 @@
         <f t="array" ref="E8">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D8),0)),NA())</f>
       </c>
       <c r="F8">
-        <f t="array" ref="F8">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D8),0)),NA())</f>
+        <f t="array" ref="F8">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D8),0)),NA())</f>
       </c>
       <c r="G8">
         <f t="array" ref="G8">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),7),NA())</f>
@@ -1396,7 +1440,7 @@
         <f t="array" ref="H8">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G8),0)),NA())</f>
       </c>
       <c r="I8">
-        <f t="array" ref="I8">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G8),0)),NA())</f>
+        <f t="array" ref="I8">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G8),0)),NA())</f>
       </c>
     </row>
     <row r="9">
@@ -1407,7 +1451,7 @@
         <f t="array" ref="B9">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A9),0)),NA())</f>
       </c>
       <c r="C9">
-        <f t="array" ref="C9">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A9),0)),NA())</f>
+        <f t="array" ref="C9">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A9),0)),NA())</f>
       </c>
       <c r="D9">
         <f t="array" ref="D9">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),8),NA())</f>
@@ -1416,7 +1460,7 @@
         <f t="array" ref="E9">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D9),0)),NA())</f>
       </c>
       <c r="F9">
-        <f t="array" ref="F9">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D9),0)),NA())</f>
+        <f t="array" ref="F9">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D9),0)),NA())</f>
       </c>
       <c r="G9">
         <f t="array" ref="G9">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),8),NA())</f>
@@ -1425,7 +1469,7 @@
         <f t="array" ref="H9">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G9),0)),NA())</f>
       </c>
       <c r="I9">
-        <f t="array" ref="I9">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G9),0)),NA())</f>
+        <f t="array" ref="I9">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G9),0)),NA())</f>
       </c>
     </row>
     <row r="10">
@@ -1436,7 +1480,7 @@
         <f t="array" ref="B10">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A10),0)),NA())</f>
       </c>
       <c r="C10">
-        <f t="array" ref="C10">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A10),0)),NA())</f>
+        <f t="array" ref="C10">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A10),0)),NA())</f>
       </c>
       <c r="D10">
         <f t="array" ref="D10">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),9),NA())</f>
@@ -1445,7 +1489,7 @@
         <f t="array" ref="E10">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D10),0)),NA())</f>
       </c>
       <c r="F10">
-        <f t="array" ref="F10">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D10),0)),NA())</f>
+        <f t="array" ref="F10">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D10),0)),NA())</f>
       </c>
       <c r="G10">
         <f t="array" ref="G10">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),9),NA())</f>
@@ -1454,7 +1498,7 @@
         <f t="array" ref="H10">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G10),0)),NA())</f>
       </c>
       <c r="I10">
-        <f t="array" ref="I10">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G10),0)),NA())</f>
+        <f t="array" ref="I10">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G10),0)),NA())</f>
       </c>
     </row>
     <row r="11">
@@ -1465,7 +1509,7 @@
         <f t="array" ref="B11">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A11),0)),NA())</f>
       </c>
       <c r="C11">
-        <f t="array" ref="C11">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A11),0)),NA())</f>
+        <f t="array" ref="C11">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A11),0)),NA())</f>
       </c>
       <c r="D11">
         <f t="array" ref="D11">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),10),NA())</f>
@@ -1474,7 +1518,7 @@
         <f t="array" ref="E11">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D11),0)),NA())</f>
       </c>
       <c r="F11">
-        <f t="array" ref="F11">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D11),0)),NA())</f>
+        <f t="array" ref="F11">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D11),0)),NA())</f>
       </c>
       <c r="G11">
         <f t="array" ref="G11">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),10),NA())</f>
@@ -1483,7 +1527,7 @@
         <f t="array" ref="H11">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G11),0)),NA())</f>
       </c>
       <c r="I11">
-        <f t="array" ref="I11">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G11),0)),NA())</f>
+        <f t="array" ref="I11">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G11),0)),NA())</f>
       </c>
     </row>
     <row r="12">
@@ -1494,7 +1538,7 @@
         <f t="array" ref="B12">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A12),0)),NA())</f>
       </c>
       <c r="C12">
-        <f t="array" ref="C12">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A12),0)),NA())</f>
+        <f t="array" ref="C12">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A12),0)),NA())</f>
       </c>
       <c r="D12">
         <f t="array" ref="D12">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),11),NA())</f>
@@ -1503,7 +1547,7 @@
         <f t="array" ref="E12">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D12),0)),NA())</f>
       </c>
       <c r="F12">
-        <f t="array" ref="F12">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D12),0)),NA())</f>
+        <f t="array" ref="F12">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D12),0)),NA())</f>
       </c>
       <c r="G12">
         <f t="array" ref="G12">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),11),NA())</f>
@@ -1512,7 +1556,7 @@
         <f t="array" ref="H12">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G12),0)),NA())</f>
       </c>
       <c r="I12">
-        <f t="array" ref="I12">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G12),0)),NA())</f>
+        <f t="array" ref="I12">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G12),0)),NA())</f>
       </c>
     </row>
     <row r="13">
@@ -1523,7 +1567,7 @@
         <f t="array" ref="B13">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A13),0)),NA())</f>
       </c>
       <c r="C13">
-        <f t="array" ref="C13">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A13),0)),NA())</f>
+        <f t="array" ref="C13">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A13),0)),NA())</f>
       </c>
       <c r="D13">
         <f t="array" ref="D13">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),12),NA())</f>
@@ -1532,7 +1576,7 @@
         <f t="array" ref="E13">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D13),0)),NA())</f>
       </c>
       <c r="F13">
-        <f t="array" ref="F13">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D13),0)),NA())</f>
+        <f t="array" ref="F13">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D13),0)),NA())</f>
       </c>
       <c r="G13">
         <f t="array" ref="G13">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),12),NA())</f>
@@ -1541,7 +1585,7 @@
         <f t="array" ref="H13">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G13),0)),NA())</f>
       </c>
       <c r="I13">
-        <f t="array" ref="I13">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G13),0)),NA())</f>
+        <f t="array" ref="I13">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G13),0)),NA())</f>
       </c>
     </row>
     <row r="14">
@@ -1552,7 +1596,7 @@
         <f t="array" ref="B14">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A14),0)),NA())</f>
       </c>
       <c r="C14">
-        <f t="array" ref="C14">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A14),0)),NA())</f>
+        <f t="array" ref="C14">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A14),0)),NA())</f>
       </c>
       <c r="D14">
         <f t="array" ref="D14">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),13),NA())</f>
@@ -1561,7 +1605,7 @@
         <f t="array" ref="E14">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D14),0)),NA())</f>
       </c>
       <c r="F14">
-        <f t="array" ref="F14">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D14),0)),NA())</f>
+        <f t="array" ref="F14">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D14),0)),NA())</f>
       </c>
       <c r="G14">
         <f t="array" ref="G14">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),13),NA())</f>
@@ -1570,7 +1614,7 @@
         <f t="array" ref="H14">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G14),0)),NA())</f>
       </c>
       <c r="I14">
-        <f t="array" ref="I14">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G14),0)),NA())</f>
+        <f t="array" ref="I14">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G14),0)),NA())</f>
       </c>
     </row>
     <row r="15">
@@ -1581,7 +1625,7 @@
         <f t="array" ref="B15">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A15),0)),NA())</f>
       </c>
       <c r="C15">
-        <f t="array" ref="C15">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A15),0)),NA())</f>
+        <f t="array" ref="C15">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A15),0)),NA())</f>
       </c>
       <c r="D15">
         <f t="array" ref="D15">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),14),NA())</f>
@@ -1590,7 +1634,7 @@
         <f t="array" ref="E15">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D15),0)),NA())</f>
       </c>
       <c r="F15">
-        <f t="array" ref="F15">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D15),0)),NA())</f>
+        <f t="array" ref="F15">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D15),0)),NA())</f>
       </c>
       <c r="G15">
         <f t="array" ref="G15">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),14),NA())</f>
@@ -1599,7 +1643,7 @@
         <f t="array" ref="H15">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G15),0)),NA())</f>
       </c>
       <c r="I15">
-        <f t="array" ref="I15">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G15),0)),NA())</f>
+        <f t="array" ref="I15">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G15),0)),NA())</f>
       </c>
     </row>
     <row r="16">
@@ -1610,7 +1654,7 @@
         <f t="array" ref="B16">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A16),0)),NA())</f>
       </c>
       <c r="C16">
-        <f t="array" ref="C16">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A16),0)),NA())</f>
+        <f t="array" ref="C16">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A16),0)),NA())</f>
       </c>
       <c r="D16">
         <f t="array" ref="D16">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),15),NA())</f>
@@ -1619,7 +1663,7 @@
         <f t="array" ref="E16">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D16),0)),NA())</f>
       </c>
       <c r="F16">
-        <f t="array" ref="F16">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D16),0)),NA())</f>
+        <f t="array" ref="F16">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D16),0)),NA())</f>
       </c>
       <c r="G16">
         <f t="array" ref="G16">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),15),NA())</f>
@@ -1628,7 +1672,7 @@
         <f t="array" ref="H16">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G16),0)),NA())</f>
       </c>
       <c r="I16">
-        <f t="array" ref="I16">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G16),0)),NA())</f>
+        <f t="array" ref="I16">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G16),0)),NA())</f>
       </c>
     </row>
     <row r="17">
@@ -1639,7 +1683,7 @@
         <f t="array" ref="B17">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A17),0)),NA())</f>
       </c>
       <c r="C17">
-        <f t="array" ref="C17">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A17),0)),NA())</f>
+        <f t="array" ref="C17">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A17),0)),NA())</f>
       </c>
       <c r="D17">
         <f t="array" ref="D17">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),16),NA())</f>
@@ -1648,7 +1692,7 @@
         <f t="array" ref="E17">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D17),0)),NA())</f>
       </c>
       <c r="F17">
-        <f t="array" ref="F17">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D17),0)),NA())</f>
+        <f t="array" ref="F17">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D17),0)),NA())</f>
       </c>
       <c r="G17">
         <f t="array" ref="G17">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),16),NA())</f>
@@ -1657,7 +1701,7 @@
         <f t="array" ref="H17">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G17),0)),NA())</f>
       </c>
       <c r="I17">
-        <f t="array" ref="I17">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G17),0)),NA())</f>
+        <f t="array" ref="I17">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G17),0)),NA())</f>
       </c>
     </row>
     <row r="18">
@@ -1668,7 +1712,7 @@
         <f t="array" ref="B18">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A18),0)),NA())</f>
       </c>
       <c r="C18">
-        <f t="array" ref="C18">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A18),0)),NA())</f>
+        <f t="array" ref="C18">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A18),0)),NA())</f>
       </c>
       <c r="D18">
         <f t="array" ref="D18">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),17),NA())</f>
@@ -1677,7 +1721,7 @@
         <f t="array" ref="E18">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D18),0)),NA())</f>
       </c>
       <c r="F18">
-        <f t="array" ref="F18">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D18),0)),NA())</f>
+        <f t="array" ref="F18">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D18),0)),NA())</f>
       </c>
       <c r="G18">
         <f t="array" ref="G18">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),17),NA())</f>
@@ -1686,7 +1730,7 @@
         <f t="array" ref="H18">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G18),0)),NA())</f>
       </c>
       <c r="I18">
-        <f t="array" ref="I18">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G18),0)),NA())</f>
+        <f t="array" ref="I18">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G18),0)),NA())</f>
       </c>
     </row>
     <row r="19">
@@ -1697,7 +1741,7 @@
         <f t="array" ref="B19">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A19),0)),NA())</f>
       </c>
       <c r="C19">
-        <f t="array" ref="C19">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A19),0)),NA())</f>
+        <f t="array" ref="C19">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A19),0)),NA())</f>
       </c>
       <c r="D19">
         <f t="array" ref="D19">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),18),NA())</f>
@@ -1706,7 +1750,7 @@
         <f t="array" ref="E19">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D19),0)),NA())</f>
       </c>
       <c r="F19">
-        <f t="array" ref="F19">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D19),0)),NA())</f>
+        <f t="array" ref="F19">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D19),0)),NA())</f>
       </c>
       <c r="G19">
         <f t="array" ref="G19">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),18),NA())</f>
@@ -1715,7 +1759,7 @@
         <f t="array" ref="H19">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G19),0)),NA())</f>
       </c>
       <c r="I19">
-        <f t="array" ref="I19">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G19),0)),NA())</f>
+        <f t="array" ref="I19">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G19),0)),NA())</f>
       </c>
     </row>
     <row r="20">
@@ -1726,7 +1770,7 @@
         <f t="array" ref="B20">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A20),0)),NA())</f>
       </c>
       <c r="C20">
-        <f t="array" ref="C20">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A20),0)),NA())</f>
+        <f t="array" ref="C20">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A20),0)),NA())</f>
       </c>
       <c r="D20">
         <f t="array" ref="D20">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),19),NA())</f>
@@ -1735,7 +1779,7 @@
         <f t="array" ref="E20">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D20),0)),NA())</f>
       </c>
       <c r="F20">
-        <f t="array" ref="F20">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D20),0)),NA())</f>
+        <f t="array" ref="F20">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D20),0)),NA())</f>
       </c>
       <c r="G20">
         <f t="array" ref="G20">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),19),NA())</f>
@@ -1744,7 +1788,7 @@
         <f t="array" ref="H20">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G20),0)),NA())</f>
       </c>
       <c r="I20">
-        <f t="array" ref="I20">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G20),0)),NA())</f>
+        <f t="array" ref="I20">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G20),0)),NA())</f>
       </c>
     </row>
     <row r="21">
@@ -1755,7 +1799,7 @@
         <f t="array" ref="B21">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A21),0)),NA())</f>
       </c>
       <c r="C21">
-        <f t="array" ref="C21">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A21),0)),NA())</f>
+        <f t="array" ref="C21">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A21),0)),NA())</f>
       </c>
       <c r="D21">
         <f t="array" ref="D21">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),20),NA())</f>
@@ -1764,7 +1808,7 @@
         <f t="array" ref="E21">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D21),0)),NA())</f>
       </c>
       <c r="F21">
-        <f t="array" ref="F21">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D21),0)),NA())</f>
+        <f t="array" ref="F21">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D21),0)),NA())</f>
       </c>
       <c r="G21">
         <f t="array" ref="G21">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),20),NA())</f>
@@ -1773,7 +1817,7 @@
         <f t="array" ref="H21">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G21),0)),NA())</f>
       </c>
       <c r="I21">
-        <f t="array" ref="I21">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G21),0)),NA())</f>
+        <f t="array" ref="I21">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G21),0)),NA())</f>
       </c>
     </row>
     <row r="22">
@@ -1784,7 +1828,7 @@
         <f t="array" ref="B22">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A22),0)),NA())</f>
       </c>
       <c r="C22">
-        <f t="array" ref="C22">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A22),0)),NA())</f>
+        <f t="array" ref="C22">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A22),0)),NA())</f>
       </c>
       <c r="D22">
         <f t="array" ref="D22">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),21),NA())</f>
@@ -1793,7 +1837,7 @@
         <f t="array" ref="E22">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D22),0)),NA())</f>
       </c>
       <c r="F22">
-        <f t="array" ref="F22">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D22),0)),NA())</f>
+        <f t="array" ref="F22">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D22),0)),NA())</f>
       </c>
       <c r="G22">
         <f t="array" ref="G22">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),21),NA())</f>
@@ -1802,7 +1846,7 @@
         <f t="array" ref="H22">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G22),0)),NA())</f>
       </c>
       <c r="I22">
-        <f t="array" ref="I22">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G22),0)),NA())</f>
+        <f t="array" ref="I22">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G22),0)),NA())</f>
       </c>
     </row>
     <row r="23">
@@ -1813,7 +1857,7 @@
         <f t="array" ref="B23">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A23),0)),NA())</f>
       </c>
       <c r="C23">
-        <f t="array" ref="C23">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A23),0)),NA())</f>
+        <f t="array" ref="C23">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A23),0)),NA())</f>
       </c>
       <c r="D23">
         <f t="array" ref="D23">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),22),NA())</f>
@@ -1822,7 +1866,7 @@
         <f t="array" ref="E23">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D23),0)),NA())</f>
       </c>
       <c r="F23">
-        <f t="array" ref="F23">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D23),0)),NA())</f>
+        <f t="array" ref="F23">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D23),0)),NA())</f>
       </c>
       <c r="G23">
         <f t="array" ref="G23">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),22),NA())</f>
@@ -1831,7 +1875,7 @@
         <f t="array" ref="H23">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G23),0)),NA())</f>
       </c>
       <c r="I23">
-        <f t="array" ref="I23">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G23),0)),NA())</f>
+        <f t="array" ref="I23">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G23),0)),NA())</f>
       </c>
     </row>
     <row r="24">
@@ -1842,7 +1886,7 @@
         <f t="array" ref="B24">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A24),0)),NA())</f>
       </c>
       <c r="C24">
-        <f t="array" ref="C24">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A24),0)),NA())</f>
+        <f t="array" ref="C24">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A24),0)),NA())</f>
       </c>
       <c r="D24">
         <f t="array" ref="D24">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),23),NA())</f>
@@ -1851,7 +1895,7 @@
         <f t="array" ref="E24">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D24),0)),NA())</f>
       </c>
       <c r="F24">
-        <f t="array" ref="F24">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D24),0)),NA())</f>
+        <f t="array" ref="F24">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D24),0)),NA())</f>
       </c>
       <c r="G24">
         <f t="array" ref="G24">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),23),NA())</f>
@@ -1860,7 +1904,7 @@
         <f t="array" ref="H24">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G24),0)),NA())</f>
       </c>
       <c r="I24">
-        <f t="array" ref="I24">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G24),0)),NA())</f>
+        <f t="array" ref="I24">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G24),0)),NA())</f>
       </c>
     </row>
     <row r="25">
@@ -1871,7 +1915,7 @@
         <f t="array" ref="B25">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A25),0)),NA())</f>
       </c>
       <c r="C25">
-        <f t="array" ref="C25">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A25),0)),NA())</f>
+        <f t="array" ref="C25">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A25),0)),NA())</f>
       </c>
       <c r="D25">
         <f t="array" ref="D25">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),24),NA())</f>
@@ -1880,7 +1924,7 @@
         <f t="array" ref="E25">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D25),0)),NA())</f>
       </c>
       <c r="F25">
-        <f t="array" ref="F25">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D25),0)),NA())</f>
+        <f t="array" ref="F25">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D25),0)),NA())</f>
       </c>
       <c r="G25">
         <f t="array" ref="G25">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),24),NA())</f>
@@ -1889,7 +1933,7 @@
         <f t="array" ref="H25">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G25),0)),NA())</f>
       </c>
       <c r="I25">
-        <f t="array" ref="I25">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G25),0)),NA())</f>
+        <f t="array" ref="I25">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G25),0)),NA())</f>
       </c>
     </row>
     <row r="26">
@@ -1900,7 +1944,7 @@
         <f t="array" ref="B26">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A26),0)),NA())</f>
       </c>
       <c r="C26">
-        <f t="array" ref="C26">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A26),0)),NA())</f>
+        <f t="array" ref="C26">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A26),0)),NA())</f>
       </c>
       <c r="D26">
         <f t="array" ref="D26">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),25),NA())</f>
@@ -1909,7 +1953,7 @@
         <f t="array" ref="E26">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D26),0)),NA())</f>
       </c>
       <c r="F26">
-        <f t="array" ref="F26">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D26),0)),NA())</f>
+        <f t="array" ref="F26">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D26),0)),NA())</f>
       </c>
       <c r="G26">
         <f t="array" ref="G26">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),25),NA())</f>
@@ -1918,7 +1962,7 @@
         <f t="array" ref="H26">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G26),0)),NA())</f>
       </c>
       <c r="I26">
-        <f t="array" ref="I26">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G26),0)),NA())</f>
+        <f t="array" ref="I26">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G26),0)),NA())</f>
       </c>
     </row>
     <row r="27">
@@ -1929,7 +1973,7 @@
         <f t="array" ref="B27">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A27),0)),NA())</f>
       </c>
       <c r="C27">
-        <f t="array" ref="C27">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A27),0)),NA())</f>
+        <f t="array" ref="C27">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A27),0)),NA())</f>
       </c>
       <c r="D27">
         <f t="array" ref="D27">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),26),NA())</f>
@@ -1938,7 +1982,7 @@
         <f t="array" ref="E27">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D27),0)),NA())</f>
       </c>
       <c r="F27">
-        <f t="array" ref="F27">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D27),0)),NA())</f>
+        <f t="array" ref="F27">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D27),0)),NA())</f>
       </c>
       <c r="G27">
         <f t="array" ref="G27">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),26),NA())</f>
@@ -1947,7 +1991,7 @@
         <f t="array" ref="H27">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G27),0)),NA())</f>
       </c>
       <c r="I27">
-        <f t="array" ref="I27">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G27),0)),NA())</f>
+        <f t="array" ref="I27">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G27),0)),NA())</f>
       </c>
     </row>
     <row r="28">
@@ -1958,7 +2002,7 @@
         <f t="array" ref="B28">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A28),0)),NA())</f>
       </c>
       <c r="C28">
-        <f t="array" ref="C28">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A28),0)),NA())</f>
+        <f t="array" ref="C28">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A28),0)),NA())</f>
       </c>
       <c r="D28">
         <f t="array" ref="D28">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),27),NA())</f>
@@ -1967,7 +2011,7 @@
         <f t="array" ref="E28">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D28),0)),NA())</f>
       </c>
       <c r="F28">
-        <f t="array" ref="F28">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D28),0)),NA())</f>
+        <f t="array" ref="F28">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D28),0)),NA())</f>
       </c>
       <c r="G28">
         <f t="array" ref="G28">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),27),NA())</f>
@@ -1976,7 +2020,7 @@
         <f t="array" ref="H28">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G28),0)),NA())</f>
       </c>
       <c r="I28">
-        <f t="array" ref="I28">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G28),0)),NA())</f>
+        <f t="array" ref="I28">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G28),0)),NA())</f>
       </c>
     </row>
     <row r="29">
@@ -1987,7 +2031,7 @@
         <f t="array" ref="B29">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A29),0)),NA())</f>
       </c>
       <c r="C29">
-        <f t="array" ref="C29">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A29),0)),NA())</f>
+        <f t="array" ref="C29">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A29),0)),NA())</f>
       </c>
       <c r="D29">
         <f t="array" ref="D29">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),28),NA())</f>
@@ -1996,7 +2040,7 @@
         <f t="array" ref="E29">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D29),0)),NA())</f>
       </c>
       <c r="F29">
-        <f t="array" ref="F29">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D29),0)),NA())</f>
+        <f t="array" ref="F29">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D29),0)),NA())</f>
       </c>
       <c r="G29">
         <f t="array" ref="G29">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),28),NA())</f>
@@ -2005,7 +2049,7 @@
         <f t="array" ref="H29">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G29),0)),NA())</f>
       </c>
       <c r="I29">
-        <f t="array" ref="I29">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G29),0)),NA())</f>
+        <f t="array" ref="I29">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G29),0)),NA())</f>
       </c>
     </row>
     <row r="30">
@@ -2016,7 +2060,7 @@
         <f t="array" ref="B30">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A30),0)),NA())</f>
       </c>
       <c r="C30">
-        <f t="array" ref="C30">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A30),0)),NA())</f>
+        <f t="array" ref="C30">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A30),0)),NA())</f>
       </c>
       <c r="D30">
         <f t="array" ref="D30">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),29),NA())</f>
@@ -2025,7 +2069,7 @@
         <f t="array" ref="E30">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D30),0)),NA())</f>
       </c>
       <c r="F30">
-        <f t="array" ref="F30">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D30),0)),NA())</f>
+        <f t="array" ref="F30">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D30),0)),NA())</f>
       </c>
       <c r="G30">
         <f t="array" ref="G30">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),29),NA())</f>
@@ -2034,7 +2078,7 @@
         <f t="array" ref="H30">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G30),0)),NA())</f>
       </c>
       <c r="I30">
-        <f t="array" ref="I30">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G30),0)),NA())</f>
+        <f t="array" ref="I30">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G30),0)),NA())</f>
       </c>
     </row>
     <row r="31">
@@ -2045,7 +2089,7 @@
         <f t="array" ref="B31">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A31),0)),NA())</f>
       </c>
       <c r="C31">
-        <f t="array" ref="C31">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A31),0)),NA())</f>
+        <f t="array" ref="C31">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A31),0)),NA())</f>
       </c>
       <c r="D31">
         <f t="array" ref="D31">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),30),NA())</f>
@@ -2054,7 +2098,7 @@
         <f t="array" ref="E31">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D31),0)),NA())</f>
       </c>
       <c r="F31">
-        <f t="array" ref="F31">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D31),0)),NA())</f>
+        <f t="array" ref="F31">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D31),0)),NA())</f>
       </c>
       <c r="G31">
         <f t="array" ref="G31">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),30),NA())</f>
@@ -2063,7 +2107,7 @@
         <f t="array" ref="H31">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G31),0)),NA())</f>
       </c>
       <c r="I31">
-        <f t="array" ref="I31">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G31),0)),NA())</f>
+        <f t="array" ref="I31">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G31),0)),NA())</f>
       </c>
     </row>
     <row r="32">
@@ -2074,7 +2118,7 @@
         <f t="array" ref="B32">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A32),0)),NA())</f>
       </c>
       <c r="C32">
-        <f t="array" ref="C32">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A32),0)),NA())</f>
+        <f t="array" ref="C32">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A32),0)),NA())</f>
       </c>
       <c r="D32">
         <f t="array" ref="D32">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),31),NA())</f>
@@ -2083,7 +2127,7 @@
         <f t="array" ref="E32">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D32),0)),NA())</f>
       </c>
       <c r="F32">
-        <f t="array" ref="F32">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D32),0)),NA())</f>
+        <f t="array" ref="F32">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D32),0)),NA())</f>
       </c>
       <c r="G32">
         <f t="array" ref="G32">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),31),NA())</f>
@@ -2092,7 +2136,7 @@
         <f t="array" ref="H32">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G32),0)),NA())</f>
       </c>
       <c r="I32">
-        <f t="array" ref="I32">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G32),0)),NA())</f>
+        <f t="array" ref="I32">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G32),0)),NA())</f>
       </c>
     </row>
     <row r="33">
@@ -2103,7 +2147,7 @@
         <f t="array" ref="B33">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A33),0)),NA())</f>
       </c>
       <c r="C33">
-        <f t="array" ref="C33">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A33),0)),NA())</f>
+        <f t="array" ref="C33">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A33),0)),NA())</f>
       </c>
       <c r="D33">
         <f t="array" ref="D33">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),32),NA())</f>
@@ -2112,7 +2156,7 @@
         <f t="array" ref="E33">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D33),0)),NA())</f>
       </c>
       <c r="F33">
-        <f t="array" ref="F33">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D33),0)),NA())</f>
+        <f t="array" ref="F33">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D33),0)),NA())</f>
       </c>
       <c r="G33">
         <f t="array" ref="G33">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),32),NA())</f>
@@ -2121,7 +2165,7 @@
         <f t="array" ref="H33">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G33),0)),NA())</f>
       </c>
       <c r="I33">
-        <f t="array" ref="I33">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G33),0)),NA())</f>
+        <f t="array" ref="I33">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G33),0)),NA())</f>
       </c>
     </row>
     <row r="34">
@@ -2132,7 +2176,7 @@
         <f t="array" ref="B34">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A34),0)),NA())</f>
       </c>
       <c r="C34">
-        <f t="array" ref="C34">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A34),0)),NA())</f>
+        <f t="array" ref="C34">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A34),0)),NA())</f>
       </c>
       <c r="D34">
         <f t="array" ref="D34">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),33),NA())</f>
@@ -2141,7 +2185,7 @@
         <f t="array" ref="E34">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D34),0)),NA())</f>
       </c>
       <c r="F34">
-        <f t="array" ref="F34">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D34),0)),NA())</f>
+        <f t="array" ref="F34">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D34),0)),NA())</f>
       </c>
       <c r="G34">
         <f t="array" ref="G34">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),33),NA())</f>
@@ -2150,7 +2194,7 @@
         <f t="array" ref="H34">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G34),0)),NA())</f>
       </c>
       <c r="I34">
-        <f t="array" ref="I34">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G34),0)),NA())</f>
+        <f t="array" ref="I34">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G34),0)),NA())</f>
       </c>
     </row>
     <row r="35">
@@ -2161,7 +2205,7 @@
         <f t="array" ref="B35">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A35),0)),NA())</f>
       </c>
       <c r="C35">
-        <f t="array" ref="C35">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A35),0)),NA())</f>
+        <f t="array" ref="C35">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A35),0)),NA())</f>
       </c>
       <c r="D35">
         <f t="array" ref="D35">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),34),NA())</f>
@@ -2170,7 +2214,7 @@
         <f t="array" ref="E35">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D35),0)),NA())</f>
       </c>
       <c r="F35">
-        <f t="array" ref="F35">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D35),0)),NA())</f>
+        <f t="array" ref="F35">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D35),0)),NA())</f>
       </c>
       <c r="G35">
         <f t="array" ref="G35">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),34),NA())</f>
@@ -2179,7 +2223,7 @@
         <f t="array" ref="H35">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G35),0)),NA())</f>
       </c>
       <c r="I35">
-        <f t="array" ref="I35">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G35),0)),NA())</f>
+        <f t="array" ref="I35">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G35),0)),NA())</f>
       </c>
     </row>
     <row r="36">
@@ -2190,7 +2234,7 @@
         <f t="array" ref="B36">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A36),0)),NA())</f>
       </c>
       <c r="C36">
-        <f t="array" ref="C36">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A36),0)),NA())</f>
+        <f t="array" ref="C36">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A36),0)),NA())</f>
       </c>
       <c r="D36">
         <f t="array" ref="D36">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),35),NA())</f>
@@ -2199,7 +2243,7 @@
         <f t="array" ref="E36">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D36),0)),NA())</f>
       </c>
       <c r="F36">
-        <f t="array" ref="F36">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D36),0)),NA())</f>
+        <f t="array" ref="F36">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D36),0)),NA())</f>
       </c>
       <c r="G36">
         <f t="array" ref="G36">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),35),NA())</f>
@@ -2208,7 +2252,7 @@
         <f t="array" ref="H36">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G36),0)),NA())</f>
       </c>
       <c r="I36">
-        <f t="array" ref="I36">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G36),0)),NA())</f>
+        <f t="array" ref="I36">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G36),0)),NA())</f>
       </c>
     </row>
     <row r="37">
@@ -2219,7 +2263,7 @@
         <f t="array" ref="B37">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A37),0)),NA())</f>
       </c>
       <c r="C37">
-        <f t="array" ref="C37">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A37),0)),NA())</f>
+        <f t="array" ref="C37">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A37),0)),NA())</f>
       </c>
       <c r="D37">
         <f t="array" ref="D37">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),36),NA())</f>
@@ -2228,7 +2272,7 @@
         <f t="array" ref="E37">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D37),0)),NA())</f>
       </c>
       <c r="F37">
-        <f t="array" ref="F37">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D37),0)),NA())</f>
+        <f t="array" ref="F37">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D37),0)),NA())</f>
       </c>
       <c r="G37">
         <f t="array" ref="G37">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),36),NA())</f>
@@ -2237,7 +2281,7 @@
         <f t="array" ref="H37">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G37),0)),NA())</f>
       </c>
       <c r="I37">
-        <f t="array" ref="I37">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G37),0)),NA())</f>
+        <f t="array" ref="I37">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G37),0)),NA())</f>
       </c>
     </row>
     <row r="38">
@@ -2248,7 +2292,7 @@
         <f t="array" ref="B38">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A38),0)),NA())</f>
       </c>
       <c r="C38">
-        <f t="array" ref="C38">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A38),0)),NA())</f>
+        <f t="array" ref="C38">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A38),0)),NA())</f>
       </c>
       <c r="D38">
         <f t="array" ref="D38">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),37),NA())</f>
@@ -2257,7 +2301,7 @@
         <f t="array" ref="E38">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D38),0)),NA())</f>
       </c>
       <c r="F38">
-        <f t="array" ref="F38">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D38),0)),NA())</f>
+        <f t="array" ref="F38">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D38),0)),NA())</f>
       </c>
       <c r="G38">
         <f t="array" ref="G38">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),37),NA())</f>
@@ -2266,7 +2310,7 @@
         <f t="array" ref="H38">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G38),0)),NA())</f>
       </c>
       <c r="I38">
-        <f t="array" ref="I38">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G38),0)),NA())</f>
+        <f t="array" ref="I38">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G38),0)),NA())</f>
       </c>
     </row>
     <row r="39">
@@ -2277,7 +2321,7 @@
         <f t="array" ref="B39">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A39),0)),NA())</f>
       </c>
       <c r="C39">
-        <f t="array" ref="C39">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A39),0)),NA())</f>
+        <f t="array" ref="C39">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A39),0)),NA())</f>
       </c>
       <c r="D39">
         <f t="array" ref="D39">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),38),NA())</f>
@@ -2286,7 +2330,7 @@
         <f t="array" ref="E39">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D39),0)),NA())</f>
       </c>
       <c r="F39">
-        <f t="array" ref="F39">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D39),0)),NA())</f>
+        <f t="array" ref="F39">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D39),0)),NA())</f>
       </c>
       <c r="G39">
         <f t="array" ref="G39">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),38),NA())</f>
@@ -2295,7 +2339,7 @@
         <f t="array" ref="H39">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G39),0)),NA())</f>
       </c>
       <c r="I39">
-        <f t="array" ref="I39">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G39),0)),NA())</f>
+        <f t="array" ref="I39">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G39),0)),NA())</f>
       </c>
     </row>
     <row r="40">
@@ -2306,7 +2350,7 @@
         <f t="array" ref="B40">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A40),0)),NA())</f>
       </c>
       <c r="C40">
-        <f t="array" ref="C40">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A40),0)),NA())</f>
+        <f t="array" ref="C40">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A40),0)),NA())</f>
       </c>
       <c r="D40">
         <f t="array" ref="D40">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),39),NA())</f>
@@ -2315,7 +2359,7 @@
         <f t="array" ref="E40">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D40),0)),NA())</f>
       </c>
       <c r="F40">
-        <f t="array" ref="F40">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D40),0)),NA())</f>
+        <f t="array" ref="F40">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D40),0)),NA())</f>
       </c>
       <c r="G40">
         <f t="array" ref="G40">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),39),NA())</f>
@@ -2324,7 +2368,7 @@
         <f t="array" ref="H40">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G40),0)),NA())</f>
       </c>
       <c r="I40">
-        <f t="array" ref="I40">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G40),0)),NA())</f>
+        <f t="array" ref="I40">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G40),0)),NA())</f>
       </c>
     </row>
     <row r="41">
@@ -2335,7 +2379,7 @@
         <f t="array" ref="B41">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A41),0)),NA())</f>
       </c>
       <c r="C41">
-        <f t="array" ref="C41">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A41),0)),NA())</f>
+        <f t="array" ref="C41">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A41),0)),NA())</f>
       </c>
       <c r="D41">
         <f t="array" ref="D41">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),40),NA())</f>
@@ -2344,7 +2388,7 @@
         <f t="array" ref="E41">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D41),0)),NA())</f>
       </c>
       <c r="F41">
-        <f t="array" ref="F41">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D41),0)),NA())</f>
+        <f t="array" ref="F41">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D41),0)),NA())</f>
       </c>
       <c r="G41">
         <f t="array" ref="G41">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),40),NA())</f>
@@ -2353,7 +2397,7 @@
         <f t="array" ref="H41">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G41),0)),NA())</f>
       </c>
       <c r="I41">
-        <f t="array" ref="I41">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G41),0)),NA())</f>
+        <f t="array" ref="I41">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G41),0)),NA())</f>
       </c>
     </row>
     <row r="42">
@@ -2364,7 +2408,7 @@
         <f t="array" ref="B42">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A42),0)),NA())</f>
       </c>
       <c r="C42">
-        <f t="array" ref="C42">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A42),0)),NA())</f>
+        <f t="array" ref="C42">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A42),0)),NA())</f>
       </c>
       <c r="D42">
         <f t="array" ref="D42">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),41),NA())</f>
@@ -2373,7 +2417,7 @@
         <f t="array" ref="E42">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D42),0)),NA())</f>
       </c>
       <c r="F42">
-        <f t="array" ref="F42">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D42),0)),NA())</f>
+        <f t="array" ref="F42">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D42),0)),NA())</f>
       </c>
       <c r="G42">
         <f t="array" ref="G42">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),41),NA())</f>
@@ -2382,7 +2426,7 @@
         <f t="array" ref="H42">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G42),0)),NA())</f>
       </c>
       <c r="I42">
-        <f t="array" ref="I42">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G42),0)),NA())</f>
+        <f t="array" ref="I42">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G42),0)),NA())</f>
       </c>
     </row>
     <row r="43">
@@ -2393,7 +2437,7 @@
         <f t="array" ref="B43">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A43),0)),NA())</f>
       </c>
       <c r="C43">
-        <f t="array" ref="C43">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A43),0)),NA())</f>
+        <f t="array" ref="C43">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A43),0)),NA())</f>
       </c>
       <c r="D43">
         <f t="array" ref="D43">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),42),NA())</f>
@@ -2402,7 +2446,7 @@
         <f t="array" ref="E43">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D43),0)),NA())</f>
       </c>
       <c r="F43">
-        <f t="array" ref="F43">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D43),0)),NA())</f>
+        <f t="array" ref="F43">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D43),0)),NA())</f>
       </c>
       <c r="G43">
         <f t="array" ref="G43">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),42),NA())</f>
@@ -2411,7 +2455,7 @@
         <f t="array" ref="H43">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G43),0)),NA())</f>
       </c>
       <c r="I43">
-        <f t="array" ref="I43">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G43),0)),NA())</f>
+        <f t="array" ref="I43">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G43),0)),NA())</f>
       </c>
     </row>
     <row r="44">
@@ -2422,7 +2466,7 @@
         <f t="array" ref="B44">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A44),0)),NA())</f>
       </c>
       <c r="C44">
-        <f t="array" ref="C44">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A44),0)),NA())</f>
+        <f t="array" ref="C44">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A44),0)),NA())</f>
       </c>
       <c r="D44">
         <f t="array" ref="D44">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),43),NA())</f>
@@ -2431,7 +2475,7 @@
         <f t="array" ref="E44">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D44),0)),NA())</f>
       </c>
       <c r="F44">
-        <f t="array" ref="F44">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D44),0)),NA())</f>
+        <f t="array" ref="F44">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D44),0)),NA())</f>
       </c>
       <c r="G44">
         <f t="array" ref="G44">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),43),NA())</f>
@@ -2440,7 +2484,7 @@
         <f t="array" ref="H44">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G44),0)),NA())</f>
       </c>
       <c r="I44">
-        <f t="array" ref="I44">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G44),0)),NA())</f>
+        <f t="array" ref="I44">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G44),0)),NA())</f>
       </c>
     </row>
     <row r="45">
@@ -2451,7 +2495,7 @@
         <f t="array" ref="B45">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A45),0)),NA())</f>
       </c>
       <c r="C45">
-        <f t="array" ref="C45">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A45),0)),NA())</f>
+        <f t="array" ref="C45">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A45),0)),NA())</f>
       </c>
       <c r="D45">
         <f t="array" ref="D45">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),44),NA())</f>
@@ -2460,7 +2504,7 @@
         <f t="array" ref="E45">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D45),0)),NA())</f>
       </c>
       <c r="F45">
-        <f t="array" ref="F45">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D45),0)),NA())</f>
+        <f t="array" ref="F45">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D45),0)),NA())</f>
       </c>
       <c r="G45">
         <f t="array" ref="G45">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),44),NA())</f>
@@ -2469,7 +2513,7 @@
         <f t="array" ref="H45">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G45),0)),NA())</f>
       </c>
       <c r="I45">
-        <f t="array" ref="I45">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G45),0)),NA())</f>
+        <f t="array" ref="I45">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G45),0)),NA())</f>
       </c>
     </row>
     <row r="46">
@@ -2480,7 +2524,7 @@
         <f t="array" ref="B46">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A46),0)),NA())</f>
       </c>
       <c r="C46">
-        <f t="array" ref="C46">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A46),0)),NA())</f>
+        <f t="array" ref="C46">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A46),0)),NA())</f>
       </c>
       <c r="D46">
         <f t="array" ref="D46">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),45),NA())</f>
@@ -2489,7 +2533,7 @@
         <f t="array" ref="E46">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D46),0)),NA())</f>
       </c>
       <c r="F46">
-        <f t="array" ref="F46">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D46),0)),NA())</f>
+        <f t="array" ref="F46">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D46),0)),NA())</f>
       </c>
       <c r="G46">
         <f t="array" ref="G46">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),45),NA())</f>
@@ -2498,7 +2542,7 @@
         <f t="array" ref="H46">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G46),0)),NA())</f>
       </c>
       <c r="I46">
-        <f t="array" ref="I46">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G46),0)),NA())</f>
+        <f t="array" ref="I46">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G46),0)),NA())</f>
       </c>
     </row>
     <row r="47">
@@ -2509,7 +2553,7 @@
         <f t="array" ref="B47">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A47),0)),NA())</f>
       </c>
       <c r="C47">
-        <f t="array" ref="C47">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A47),0)),NA())</f>
+        <f t="array" ref="C47">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A47),0)),NA())</f>
       </c>
       <c r="D47">
         <f t="array" ref="D47">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),46),NA())</f>
@@ -2518,7 +2562,7 @@
         <f t="array" ref="E47">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D47),0)),NA())</f>
       </c>
       <c r="F47">
-        <f t="array" ref="F47">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D47),0)),NA())</f>
+        <f t="array" ref="F47">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D47),0)),NA())</f>
       </c>
       <c r="G47">
         <f t="array" ref="G47">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),46),NA())</f>
@@ -2527,7 +2571,7 @@
         <f t="array" ref="H47">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G47),0)),NA())</f>
       </c>
       <c r="I47">
-        <f t="array" ref="I47">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G47),0)),NA())</f>
+        <f t="array" ref="I47">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G47),0)),NA())</f>
       </c>
     </row>
     <row r="48">
@@ -2538,7 +2582,7 @@
         <f t="array" ref="B48">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A48),0)),NA())</f>
       </c>
       <c r="C48">
-        <f t="array" ref="C48">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A48),0)),NA())</f>
+        <f t="array" ref="C48">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A48),0)),NA())</f>
       </c>
       <c r="D48">
         <f t="array" ref="D48">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),47),NA())</f>
@@ -2547,7 +2591,7 @@
         <f t="array" ref="E48">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D48),0)),NA())</f>
       </c>
       <c r="F48">
-        <f t="array" ref="F48">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D48),0)),NA())</f>
+        <f t="array" ref="F48">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D48),0)),NA())</f>
       </c>
       <c r="G48">
         <f t="array" ref="G48">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),47),NA())</f>
@@ -2556,7 +2600,7 @@
         <f t="array" ref="H48">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G48),0)),NA())</f>
       </c>
       <c r="I48">
-        <f t="array" ref="I48">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G48),0)),NA())</f>
+        <f t="array" ref="I48">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G48),0)),NA())</f>
       </c>
     </row>
     <row r="49">
@@ -2567,7 +2611,7 @@
         <f t="array" ref="B49">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A49),0)),NA())</f>
       </c>
       <c r="C49">
-        <f t="array" ref="C49">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A49),0)),NA())</f>
+        <f t="array" ref="C49">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A49),0)),NA())</f>
       </c>
       <c r="D49">
         <f t="array" ref="D49">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),48),NA())</f>
@@ -2576,7 +2620,7 @@
         <f t="array" ref="E49">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D49),0)),NA())</f>
       </c>
       <c r="F49">
-        <f t="array" ref="F49">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D49),0)),NA())</f>
+        <f t="array" ref="F49">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D49),0)),NA())</f>
       </c>
       <c r="G49">
         <f t="array" ref="G49">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),48),NA())</f>
@@ -2585,7 +2629,7 @@
         <f t="array" ref="H49">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G49),0)),NA())</f>
       </c>
       <c r="I49">
-        <f t="array" ref="I49">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G49),0)),NA())</f>
+        <f t="array" ref="I49">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G49),0)),NA())</f>
       </c>
     </row>
     <row r="50">
@@ -2596,7 +2640,7 @@
         <f t="array" ref="B50">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A50),0)),NA())</f>
       </c>
       <c r="C50">
-        <f t="array" ref="C50">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A50),0)),NA())</f>
+        <f t="array" ref="C50">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A50),0)),NA())</f>
       </c>
       <c r="D50">
         <f t="array" ref="D50">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),49),NA())</f>
@@ -2605,7 +2649,7 @@
         <f t="array" ref="E50">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D50),0)),NA())</f>
       </c>
       <c r="F50">
-        <f t="array" ref="F50">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D50),0)),NA())</f>
+        <f t="array" ref="F50">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D50),0)),NA())</f>
       </c>
       <c r="G50">
         <f t="array" ref="G50">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),49),NA())</f>
@@ -2614,7 +2658,7 @@
         <f t="array" ref="H50">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G50),0)),NA())</f>
       </c>
       <c r="I50">
-        <f t="array" ref="I50">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G50),0)),NA())</f>
+        <f t="array" ref="I50">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G50),0)),NA())</f>
       </c>
     </row>
     <row r="51">
@@ -2625,7 +2669,7 @@
         <f t="array" ref="B51">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A51),0)),NA())</f>
       </c>
       <c r="C51">
-        <f t="array" ref="C51">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A51),0)),NA())</f>
+        <f t="array" ref="C51">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A51),0)),NA())</f>
       </c>
       <c r="D51">
         <f t="array" ref="D51">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),50),NA())</f>
@@ -2634,7 +2678,7 @@
         <f t="array" ref="E51">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D51),0)),NA())</f>
       </c>
       <c r="F51">
-        <f t="array" ref="F51">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D51),0)),NA())</f>
+        <f t="array" ref="F51">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D51),0)),NA())</f>
       </c>
       <c r="G51">
         <f t="array" ref="G51">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),50),NA())</f>
@@ -2643,7 +2687,7 @@
         <f t="array" ref="H51">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G51),0)),NA())</f>
       </c>
       <c r="I51">
-        <f t="array" ref="I51">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G51),0)),NA())</f>
+        <f t="array" ref="I51">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G51),0)),NA())</f>
       </c>
     </row>
     <row r="52">
@@ -2654,7 +2698,7 @@
         <f t="array" ref="B52">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A52),0)),NA())</f>
       </c>
       <c r="C52">
-        <f t="array" ref="C52">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A52),0)),NA())</f>
+        <f t="array" ref="C52">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A52),0)),NA())</f>
       </c>
       <c r="D52">
         <f t="array" ref="D52">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),51),NA())</f>
@@ -2663,7 +2707,7 @@
         <f t="array" ref="E52">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D52),0)),NA())</f>
       </c>
       <c r="F52">
-        <f t="array" ref="F52">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D52),0)),NA())</f>
+        <f t="array" ref="F52">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D52),0)),NA())</f>
       </c>
       <c r="G52">
         <f t="array" ref="G52">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),51),NA())</f>
@@ -2672,7 +2716,7 @@
         <f t="array" ref="H52">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G52),0)),NA())</f>
       </c>
       <c r="I52">
-        <f t="array" ref="I52">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G52),0)),NA())</f>
+        <f t="array" ref="I52">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G52),0)),NA())</f>
       </c>
     </row>
     <row r="53">
@@ -2683,7 +2727,7 @@
         <f t="array" ref="B53">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A53),0)),NA())</f>
       </c>
       <c r="C53">
-        <f t="array" ref="C53">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A53),0)),NA())</f>
+        <f t="array" ref="C53">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A53),0)),NA())</f>
       </c>
       <c r="D53">
         <f t="array" ref="D53">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),52),NA())</f>
@@ -2692,7 +2736,7 @@
         <f t="array" ref="E53">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D53),0)),NA())</f>
       </c>
       <c r="F53">
-        <f t="array" ref="F53">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D53),0)),NA())</f>
+        <f t="array" ref="F53">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D53),0)),NA())</f>
       </c>
       <c r="G53">
         <f t="array" ref="G53">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),52),NA())</f>
@@ -2701,7 +2745,7 @@
         <f t="array" ref="H53">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G53),0)),NA())</f>
       </c>
       <c r="I53">
-        <f t="array" ref="I53">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G53),0)),NA())</f>
+        <f t="array" ref="I53">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G53),0)),NA())</f>
       </c>
     </row>
     <row r="54">
@@ -2712,7 +2756,7 @@
         <f t="array" ref="B54">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A54),0)),NA())</f>
       </c>
       <c r="C54">
-        <f t="array" ref="C54">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A54),0)),NA())</f>
+        <f t="array" ref="C54">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A54),0)),NA())</f>
       </c>
       <c r="D54">
         <f t="array" ref="D54">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),53),NA())</f>
@@ -2721,7 +2765,7 @@
         <f t="array" ref="E54">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D54),0)),NA())</f>
       </c>
       <c r="F54">
-        <f t="array" ref="F54">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D54),0)),NA())</f>
+        <f t="array" ref="F54">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D54),0)),NA())</f>
       </c>
       <c r="G54">
         <f t="array" ref="G54">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),53),NA())</f>
@@ -2730,7 +2774,7 @@
         <f t="array" ref="H54">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G54),0)),NA())</f>
       </c>
       <c r="I54">
-        <f t="array" ref="I54">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G54),0)),NA())</f>
+        <f t="array" ref="I54">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G54),0)),NA())</f>
       </c>
     </row>
     <row r="55">
@@ -2741,7 +2785,7 @@
         <f t="array" ref="B55">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A55),0)),NA())</f>
       </c>
       <c r="C55">
-        <f t="array" ref="C55">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A55),0)),NA())</f>
+        <f t="array" ref="C55">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A55),0)),NA())</f>
       </c>
       <c r="D55">
         <f t="array" ref="D55">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),54),NA())</f>
@@ -2750,7 +2794,7 @@
         <f t="array" ref="E55">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D55),0)),NA())</f>
       </c>
       <c r="F55">
-        <f t="array" ref="F55">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D55),0)),NA())</f>
+        <f t="array" ref="F55">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D55),0)),NA())</f>
       </c>
       <c r="G55">
         <f t="array" ref="G55">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),54),NA())</f>
@@ -2759,7 +2803,7 @@
         <f t="array" ref="H55">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G55),0)),NA())</f>
       </c>
       <c r="I55">
-        <f t="array" ref="I55">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G55),0)),NA())</f>
+        <f t="array" ref="I55">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G55),0)),NA())</f>
       </c>
     </row>
     <row r="56">
@@ -2770,7 +2814,7 @@
         <f t="array" ref="B56">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A56),0)),NA())</f>
       </c>
       <c r="C56">
-        <f t="array" ref="C56">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A56),0)),NA())</f>
+        <f t="array" ref="C56">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A56),0)),NA())</f>
       </c>
       <c r="D56">
         <f t="array" ref="D56">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),55),NA())</f>
@@ -2779,7 +2823,7 @@
         <f t="array" ref="E56">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D56),0)),NA())</f>
       </c>
       <c r="F56">
-        <f t="array" ref="F56">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D56),0)),NA())</f>
+        <f t="array" ref="F56">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D56),0)),NA())</f>
       </c>
       <c r="G56">
         <f t="array" ref="G56">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),55),NA())</f>
@@ -2788,7 +2832,7 @@
         <f t="array" ref="H56">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G56),0)),NA())</f>
       </c>
       <c r="I56">
-        <f t="array" ref="I56">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G56),0)),NA())</f>
+        <f t="array" ref="I56">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G56),0)),NA())</f>
       </c>
     </row>
     <row r="57">
@@ -2799,7 +2843,7 @@
         <f t="array" ref="B57">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A57),0)),NA())</f>
       </c>
       <c r="C57">
-        <f t="array" ref="C57">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A57),0)),NA())</f>
+        <f t="array" ref="C57">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A57),0)),NA())</f>
       </c>
       <c r="D57">
         <f t="array" ref="D57">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),56),NA())</f>
@@ -2808,7 +2852,7 @@
         <f t="array" ref="E57">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D57),0)),NA())</f>
       </c>
       <c r="F57">
-        <f t="array" ref="F57">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D57),0)),NA())</f>
+        <f t="array" ref="F57">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D57),0)),NA())</f>
       </c>
       <c r="G57">
         <f t="array" ref="G57">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),56),NA())</f>
@@ -2817,7 +2861,7 @@
         <f t="array" ref="H57">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G57),0)),NA())</f>
       </c>
       <c r="I57">
-        <f t="array" ref="I57">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G57),0)),NA())</f>
+        <f t="array" ref="I57">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G57),0)),NA())</f>
       </c>
     </row>
     <row r="58">
@@ -2828,7 +2872,7 @@
         <f t="array" ref="B58">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A58),0)),NA())</f>
       </c>
       <c r="C58">
-        <f t="array" ref="C58">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A58),0)),NA())</f>
+        <f t="array" ref="C58">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A58),0)),NA())</f>
       </c>
       <c r="D58">
         <f t="array" ref="D58">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),57),NA())</f>
@@ -2837,7 +2881,7 @@
         <f t="array" ref="E58">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D58),0)),NA())</f>
       </c>
       <c r="F58">
-        <f t="array" ref="F58">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D58),0)),NA())</f>
+        <f t="array" ref="F58">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D58),0)),NA())</f>
       </c>
       <c r="G58">
         <f t="array" ref="G58">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),57),NA())</f>
@@ -2846,7 +2890,7 @@
         <f t="array" ref="H58">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G58),0)),NA())</f>
       </c>
       <c r="I58">
-        <f t="array" ref="I58">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G58),0)),NA())</f>
+        <f t="array" ref="I58">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G58),0)),NA())</f>
       </c>
     </row>
     <row r="59">
@@ -2857,7 +2901,7 @@
         <f t="array" ref="B59">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A59),0)),NA())</f>
       </c>
       <c r="C59">
-        <f t="array" ref="C59">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A59),0)),NA())</f>
+        <f t="array" ref="C59">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A59),0)),NA())</f>
       </c>
       <c r="D59">
         <f t="array" ref="D59">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),58),NA())</f>
@@ -2866,7 +2910,7 @@
         <f t="array" ref="E59">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D59),0)),NA())</f>
       </c>
       <c r="F59">
-        <f t="array" ref="F59">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D59),0)),NA())</f>
+        <f t="array" ref="F59">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D59),0)),NA())</f>
       </c>
       <c r="G59">
         <f t="array" ref="G59">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),58),NA())</f>
@@ -2875,7 +2919,7 @@
         <f t="array" ref="H59">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G59),0)),NA())</f>
       </c>
       <c r="I59">
-        <f t="array" ref="I59">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G59),0)),NA())</f>
+        <f t="array" ref="I59">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G59),0)),NA())</f>
       </c>
     </row>
     <row r="60">
@@ -2886,7 +2930,7 @@
         <f t="array" ref="B60">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A60),0)),NA())</f>
       </c>
       <c r="C60">
-        <f t="array" ref="C60">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A60),0)),NA())</f>
+        <f t="array" ref="C60">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A60),0)),NA())</f>
       </c>
       <c r="D60">
         <f t="array" ref="D60">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),59),NA())</f>
@@ -2895,7 +2939,7 @@
         <f t="array" ref="E60">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D60),0)),NA())</f>
       </c>
       <c r="F60">
-        <f t="array" ref="F60">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D60),0)),NA())</f>
+        <f t="array" ref="F60">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D60),0)),NA())</f>
       </c>
       <c r="G60">
         <f t="array" ref="G60">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),59),NA())</f>
@@ -2904,7 +2948,7 @@
         <f t="array" ref="H60">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G60),0)),NA())</f>
       </c>
       <c r="I60">
-        <f t="array" ref="I60">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G60),0)),NA())</f>
+        <f t="array" ref="I60">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G60),0)),NA())</f>
       </c>
     </row>
     <row r="61">
@@ -2915,7 +2959,7 @@
         <f t="array" ref="B61">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A61),0)),NA())</f>
       </c>
       <c r="C61">
-        <f t="array" ref="C61">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A61),0)),NA())</f>
+        <f t="array" ref="C61">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=4)*('射擊表'!$B$2:$B$500=A61),0)),NA())</f>
       </c>
       <c r="D61">
         <f t="array" ref="D61">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=5,'射擊表'!$B$2:$B$500),60),NA())</f>
@@ -2924,7 +2968,7 @@
         <f t="array" ref="E61">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D61),0)),NA())</f>
       </c>
       <c r="F61">
-        <f t="array" ref="F61">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D61),0)),NA())</f>
+        <f t="array" ref="F61">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=5)*('射擊表'!$B$2:$B$500=D61),0)),NA())</f>
       </c>
       <c r="G61">
         <f t="array" ref="G61">IFERROR(SMALL(IF('射擊表'!$A$2:$A$500=6,'射擊表'!$B$2:$B$500),60),NA())</f>
@@ -2933,7 +2977,7 @@
         <f t="array" ref="H61">IFERROR(INDEX('射擊表'!$C$2:$C$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G61),0)),NA())</f>
       </c>
       <c r="I61">
-        <f t="array" ref="I61">IFERROR(INDEX('射擊表'!$D$2:$D$500,MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G61),0)),NA())</f>
+        <f t="array" ref="I61">IFERROR(INDEX(IF('射擊表'!$E$2:$E$500="us",ABS('射擊表'!$D$2:$D$500-1500)/5,'射擊表'!$D$2:$D$500),MATCH(1,('射擊表'!$A$2:$A$500=6)*('射擊表'!$B$2:$B$500=G61),0)),NA())</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bonus holes selectable (Q W E = holes 10-12), shot table holes 10-12, big Dashboard target board with elevation / flywheel / distance beside it
- OperatorTarget: Dashboard holes 10/11/12 -> Orin vision ids 1/2/3.
- CH3: 1000 + 80*k for k = 0..12 (was 100*k for 0..9); TGT,<0..12>.
  Flash the Mega and the ground STM32 together; the bridge image is unchanged.
- Shot table: Excel 洞口 1-12, HOLE_POINTS[13]; a bonus hole uses only its
  own points (no row-center fallback). shot_table.xlsx validation and help
  text updated in place, data unchanged.
- Dashboard: new top "Target / 目標洞" panel -- bonus row Q W E over the
  3x3 grid, selected hole blue, the camera's current hole green, large
  elevation / Falcon / distance readouts beside it; S records bonus points.
- Orin side (accept ids 1-3, predicted position when out of view, all
  detected holes) is the next step, per Jeremy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/shot_table/shot_table.xlsx
+++ b/tools/shot_table/shot_table.xlsx
@@ -1010,9 +1010,9 @@
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="洞口" error="洞口要是 1–9 的整數" sqref="A2:A500">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="洞口" error="洞口要是 1–12 的整數（10–12 是加分框左中右）" sqref="A2:A500">
       <formula1>1</formula1>
-      <formula2>9</formula2>
+      <formula2>12</formula2>
     </dataValidation>
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="距離" error="距離 0.5–15 m" sqref="B2:B500">
       <formula1>0.5</formula1>
@@ -1098,7 +1098,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- 洞口：Dashboard 的編號 1–9（1 左下、2 左中、3 左上 … 9 右上）。</t>
+          <t>- 洞口：Dashboard 的編號 1–9（1 左下、2 左中、3 左上 … 9 右上）；10、11、12 是最上面的加分框左、中、右（Dashboard 按 Q、W、E 選）。</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- 會借用同一排中間洞的值：1、7 用 4，2、8 用 5，3、9 用 6。</t>
+          <t>- 會借用同一排中間洞的值：1、7 用 4，2、8 用 5，3、9 用 6。加分框（10–12）不借用：沒有資料就不會對它發射。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shot table: the 26 points logged on 10-28 (holes 4/5/6) replace the old 2.50 / 5.00 m rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/shot_table/shot_table.xlsx
+++ b/tools/shot_table/shot_table.xlsx
@@ -899,13 +899,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>2.5</v>
+        <v>2.85</v>
       </c>
       <c r="C2">
-        <v>2407</v>
+        <v>500</v>
       </c>
       <c r="D2">
-        <v>42.0</v>
+        <v>37</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -918,13 +918,13 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>5.0</v>
+        <v>3.26</v>
       </c>
       <c r="C3">
-        <v>2183</v>
+        <v>500</v>
       </c>
       <c r="D3">
-        <v>43.0</v>
+        <v>37</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -934,16 +934,16 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4">
-        <v>2.5</v>
+        <v>3.66</v>
       </c>
       <c r="C4">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="D4">
-        <v>100.0</v>
+        <v>38</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -953,16 +953,16 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
-        <v>5.0</v>
+        <v>4.1</v>
       </c>
       <c r="C5">
-        <v>2063</v>
+        <v>608</v>
       </c>
       <c r="D5">
-        <v>46.0</v>
+        <v>38</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -972,16 +972,16 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6">
-        <v>2.5</v>
+        <v>4.44</v>
       </c>
       <c r="C6">
-        <v>1010</v>
+        <v>500</v>
       </c>
       <c r="D6">
-        <v>100.0</v>
+        <v>41</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -991,18 +991,398 @@
     </row>
     <row r="7">
       <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>5.12</v>
+      </c>
+      <c r="C7">
+        <v>500</v>
+      </c>
+      <c r="D7">
+        <v>42</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>5.48</v>
+      </c>
+      <c r="C8">
+        <v>500</v>
+      </c>
+      <c r="D8">
+        <v>42</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>5.9</v>
+      </c>
+      <c r="C9">
+        <v>500</v>
+      </c>
+      <c r="D9">
+        <v>44</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>4</v>
+      </c>
+      <c r="B10">
+        <v>6.36</v>
+      </c>
+      <c r="C10">
+        <v>500</v>
+      </c>
+      <c r="D10">
+        <v>47</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11">
+        <v>6.75</v>
+      </c>
+      <c r="C11">
+        <v>500</v>
+      </c>
+      <c r="D11">
+        <v>48</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>7.32</v>
+      </c>
+      <c r="C12">
+        <v>500</v>
+      </c>
+      <c r="D12">
+        <v>49</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>5</v>
+      </c>
+      <c r="B13">
+        <v>7.49</v>
+      </c>
+      <c r="C13">
+        <v>500</v>
+      </c>
+      <c r="D13">
+        <v>55</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14">
+        <v>6.82</v>
+      </c>
+      <c r="C14">
+        <v>500</v>
+      </c>
+      <c r="D14">
+        <v>53</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>6.44</v>
+      </c>
+      <c r="C15">
+        <v>500</v>
+      </c>
+      <c r="D15">
+        <v>52</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>6.22</v>
+      </c>
+      <c r="C16">
+        <v>500</v>
+      </c>
+      <c r="D16">
+        <v>51</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>5</v>
+      </c>
+      <c r="B17">
+        <v>5.75</v>
+      </c>
+      <c r="C17">
+        <v>500</v>
+      </c>
+      <c r="D17">
+        <v>50</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>5</v>
+      </c>
+      <c r="B18">
+        <v>5.32</v>
+      </c>
+      <c r="C18">
+        <v>500</v>
+      </c>
+      <c r="D18">
+        <v>49</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>5</v>
+      </c>
+      <c r="B19">
+        <v>4.98</v>
+      </c>
+      <c r="C19">
+        <v>500</v>
+      </c>
+      <c r="D19">
+        <v>48</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>5</v>
+      </c>
+      <c r="B20">
+        <v>4.6</v>
+      </c>
+      <c r="C20">
+        <v>500</v>
+      </c>
+      <c r="D20">
+        <v>48</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>5</v>
+      </c>
+      <c r="B21">
+        <v>4.41</v>
+      </c>
+      <c r="C21">
+        <v>500</v>
+      </c>
+      <c r="D21">
+        <v>48</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>5</v>
+      </c>
+      <c r="B22">
+        <v>3.99</v>
+      </c>
+      <c r="C22">
+        <v>500</v>
+      </c>
+      <c r="D22">
+        <v>47</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>5</v>
+      </c>
+      <c r="B23">
+        <v>3.55</v>
+      </c>
+      <c r="C23">
+        <v>604</v>
+      </c>
+      <c r="D23">
+        <v>46</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>5</v>
+      </c>
+      <c r="B24">
+        <v>3.1</v>
+      </c>
+      <c r="C24">
+        <v>604</v>
+      </c>
+      <c r="D24">
+        <v>47</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>5.0</v>
-      </c>
-      <c r="C7">
-        <v>2442</v>
-      </c>
-      <c r="D7">
-        <v>80.0</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="B25">
+        <v>3.87</v>
+      </c>
+      <c r="C25">
+        <v>1220</v>
+      </c>
+      <c r="D25">
+        <v>65</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>6</v>
+      </c>
+      <c r="B26">
+        <v>4.42</v>
+      </c>
+      <c r="C26">
+        <v>1036</v>
+      </c>
+      <c r="D26">
+        <v>65</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>6</v>
+      </c>
+      <c r="B27">
+        <v>4.7</v>
+      </c>
+      <c r="C27">
+        <v>865</v>
+      </c>
+      <c r="D27">
+        <v>65</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>%</t>
         </is>

</xml_diff>

<commit_message>
Shot table: the 24 points logged on 10-31 replace the 10-28 rows (flywheel values ran 7-12 points lower today)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/shot_table/shot_table.xlsx
+++ b/tools/shot_table/shot_table.xlsx
@@ -899,13 +899,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>2.85</v>
+        <v>2.72</v>
       </c>
       <c r="C2">
         <v>500</v>
       </c>
       <c r="D2">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -918,13 +918,13 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>3.26</v>
+        <v>3.3</v>
       </c>
       <c r="C3">
         <v>500</v>
       </c>
       <c r="D3">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -937,13 +937,13 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
       <c r="C4">
         <v>500</v>
       </c>
       <c r="D4">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -956,13 +956,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>608</v>
+        <v>500</v>
       </c>
       <c r="D5">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>4.44</v>
+        <v>4.48</v>
       </c>
       <c r="C6">
         <v>500</v>
       </c>
       <c r="D6">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -994,13 +994,13 @@
         <v>4</v>
       </c>
       <c r="B7">
-        <v>5.12</v>
+        <v>5.11</v>
       </c>
       <c r="C7">
         <v>500</v>
       </c>
       <c r="D7">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1013,13 +1013,13 @@
         <v>4</v>
       </c>
       <c r="B8">
-        <v>5.48</v>
+        <v>5.54</v>
       </c>
       <c r="C8">
         <v>500</v>
       </c>
       <c r="D8">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1032,13 +1032,13 @@
         <v>4</v>
       </c>
       <c r="B9">
-        <v>5.9</v>
+        <v>6.04</v>
       </c>
       <c r="C9">
         <v>500</v>
       </c>
       <c r="D9">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1051,13 +1051,13 @@
         <v>4</v>
       </c>
       <c r="B10">
-        <v>6.36</v>
+        <v>6.46</v>
       </c>
       <c r="C10">
         <v>500</v>
       </c>
       <c r="D10">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1070,13 +1070,13 @@
         <v>4</v>
       </c>
       <c r="B11">
-        <v>6.75</v>
+        <v>6.82</v>
       </c>
       <c r="C11">
         <v>500</v>
       </c>
       <c r="D11">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1086,16 +1086,16 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12">
-        <v>7.32</v>
+        <v>7.01</v>
       </c>
       <c r="C12">
         <v>500</v>
       </c>
       <c r="D12">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1108,13 +1108,13 @@
         <v>5</v>
       </c>
       <c r="B13">
-        <v>7.49</v>
+        <v>6.47</v>
       </c>
       <c r="C13">
         <v>500</v>
       </c>
       <c r="D13">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1127,13 +1127,13 @@
         <v>5</v>
       </c>
       <c r="B14">
-        <v>6.82</v>
+        <v>5.85</v>
       </c>
       <c r="C14">
         <v>500</v>
       </c>
       <c r="D14">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1146,13 +1146,13 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>6.44</v>
+        <v>5.19</v>
       </c>
       <c r="C15">
         <v>500</v>
       </c>
       <c r="D15">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1165,13 +1165,13 @@
         <v>5</v>
       </c>
       <c r="B16">
-        <v>6.22</v>
+        <v>4.29</v>
       </c>
       <c r="C16">
         <v>500</v>
       </c>
       <c r="D16">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1184,13 +1184,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>5.75</v>
+        <v>3.55</v>
       </c>
       <c r="C17">
-        <v>500</v>
+        <v>655</v>
       </c>
       <c r="D17">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1203,13 +1203,13 @@
         <v>5</v>
       </c>
       <c r="B18">
-        <v>5.32</v>
+        <v>3.23</v>
       </c>
       <c r="C18">
-        <v>500</v>
+        <v>782</v>
       </c>
       <c r="D18">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1222,13 +1222,13 @@
         <v>5</v>
       </c>
       <c r="B19">
-        <v>4.98</v>
+        <v>2.92</v>
       </c>
       <c r="C19">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="D19">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1238,16 +1238,16 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B20">
-        <v>4.6</v>
+        <v>3.25</v>
       </c>
       <c r="C20">
-        <v>500</v>
+        <v>1913</v>
       </c>
       <c r="D20">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1257,16 +1257,16 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B21">
-        <v>4.41</v>
+        <v>3.93</v>
       </c>
       <c r="C21">
-        <v>500</v>
+        <v>1378</v>
       </c>
       <c r="D21">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1276,16 +1276,16 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B22">
-        <v>3.99</v>
+        <v>4.72</v>
       </c>
       <c r="C22">
-        <v>500</v>
+        <v>973</v>
       </c>
       <c r="D22">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1295,16 +1295,16 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B23">
-        <v>3.55</v>
+        <v>5.44</v>
       </c>
       <c r="C23">
-        <v>604</v>
+        <v>560</v>
       </c>
       <c r="D23">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1314,16 +1314,16 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B24">
-        <v>3.1</v>
+        <v>6.32</v>
       </c>
       <c r="C24">
-        <v>604</v>
+        <v>500</v>
       </c>
       <c r="D24">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1336,53 +1336,15 @@
         <v>6</v>
       </c>
       <c r="B25">
-        <v>3.87</v>
+        <v>6.78</v>
       </c>
       <c r="C25">
-        <v>1220</v>
+        <v>500</v>
       </c>
       <c r="D25">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E25" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26">
-        <v>6</v>
-      </c>
-      <c r="B26">
-        <v>4.42</v>
-      </c>
-      <c r="C26">
-        <v>1036</v>
-      </c>
-      <c r="D26">
-        <v>65</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27">
-        <v>6</v>
-      </c>
-      <c r="B27">
-        <v>4.7</v>
-      </c>
-      <c r="C27">
-        <v>865</v>
-      </c>
-      <c r="D27">
-        <v>65</v>
-      </c>
-      <c r="E27" t="inlineStr">
         <is>
           <t>%</t>
         </is>

</xml_diff>

<commit_message>
Bonus holes borrow like the other rows: Q / E (10 / 12) use W (11) when they have no points; apply.py FALLBACK, Excel help rebuilt (same points)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/shot_table/shot_table.xlsx
+++ b/tools/shot_table/shot_table.xlsx
@@ -905,7 +905,7 @@
         <v>500</v>
       </c>
       <c r="D2">
-        <v>32</v>
+        <v>32.0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         <v>500</v>
       </c>
       <c r="D3">
-        <v>32</v>
+        <v>32.0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         <v>500</v>
       </c>
       <c r="D4">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -956,13 +956,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>4.0</v>
       </c>
       <c r="C5">
         <v>500</v>
       </c>
       <c r="D5">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -981,7 +981,7 @@
         <v>500</v>
       </c>
       <c r="D6">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>500</v>
       </c>
       <c r="D7">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
         <v>500</v>
       </c>
       <c r="D8">
-        <v>36</v>
+        <v>36.0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
         <v>500</v>
       </c>
       <c r="D9">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
         <v>500</v>
       </c>
       <c r="D10">
-        <v>38</v>
+        <v>38.0</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
         <v>500</v>
       </c>
       <c r="D11">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1089,13 +1089,13 @@
         <v>5</v>
       </c>
       <c r="B12">
-        <v>7.01</v>
+        <v>2.92</v>
       </c>
       <c r="C12">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="D12">
-        <v>40</v>
+        <v>36.0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1108,13 +1108,13 @@
         <v>5</v>
       </c>
       <c r="B13">
-        <v>6.47</v>
+        <v>3.23</v>
       </c>
       <c r="C13">
-        <v>500</v>
+        <v>782</v>
       </c>
       <c r="D13">
-        <v>39</v>
+        <v>36.0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1127,13 +1127,13 @@
         <v>5</v>
       </c>
       <c r="B14">
-        <v>5.85</v>
+        <v>3.55</v>
       </c>
       <c r="C14">
-        <v>500</v>
+        <v>655</v>
       </c>
       <c r="D14">
-        <v>38</v>
+        <v>36.0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1146,13 +1146,13 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>5.19</v>
+        <v>4.29</v>
       </c>
       <c r="C15">
         <v>500</v>
       </c>
       <c r="D15">
-        <v>37</v>
+        <v>36.0</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1165,13 +1165,13 @@
         <v>5</v>
       </c>
       <c r="B16">
-        <v>4.29</v>
+        <v>5.19</v>
       </c>
       <c r="C16">
         <v>500</v>
       </c>
       <c r="D16">
-        <v>36</v>
+        <v>37.0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1184,13 +1184,13 @@
         <v>5</v>
       </c>
       <c r="B17">
-        <v>3.55</v>
+        <v>5.85</v>
       </c>
       <c r="C17">
-        <v>655</v>
+        <v>500</v>
       </c>
       <c r="D17">
-        <v>36</v>
+        <v>38.0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1203,13 +1203,13 @@
         <v>5</v>
       </c>
       <c r="B18">
-        <v>3.23</v>
+        <v>6.47</v>
       </c>
       <c r="C18">
-        <v>782</v>
+        <v>500</v>
       </c>
       <c r="D18">
-        <v>36</v>
+        <v>39.0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1222,13 +1222,13 @@
         <v>5</v>
       </c>
       <c r="B19">
-        <v>2.92</v>
+        <v>7.01</v>
       </c>
       <c r="C19">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="D19">
-        <v>36</v>
+        <v>40.0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         <v>1913</v>
       </c>
       <c r="D20">
-        <v>60</v>
+        <v>60.0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
         <v>1378</v>
       </c>
       <c r="D21">
-        <v>60</v>
+        <v>60.0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>973</v>
       </c>
       <c r="D22">
-        <v>60</v>
+        <v>60.0</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1304,7 +1304,7 @@
         <v>560</v>
       </c>
       <c r="D23">
-        <v>60</v>
+        <v>60.0</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         <v>500</v>
       </c>
       <c r="D24">
-        <v>68</v>
+        <v>68.0</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>500</v>
       </c>
       <c r="D25">
-        <v>68</v>
+        <v>68.0</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1416,113 +1416,127 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>格式（嚴格）</t>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3. Dashboard 按 S 記錄的點：在 Dashboard 按「下載 CSV」，關掉 Excel，執行 python3 tools/shot_table/apply.py --import --upload（同洞口同距離會取代，其他加在最後）。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- 第 1 列是欄位名稱。「洞口」「距離(m)」「仰角(us)」「轉速」「轉速單位」五個必須各出現一次、名稱一字不差。</t>
+          <t>格式（嚴格）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>- 若插入其他欄位，新欄位一定要有名稱；它們不會被讀取。</t>
+          <t>- 第 1 列是欄位名稱。「洞口」「距離(m)」「仰角(us)」「轉速」「轉速單位」五個必須各出現一次、名稱一字不差。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- 洞口：Dashboard 的編號 1–9（1 左下、2 左中、3 左上 … 9 右上）；10、11、12 是最上面的加分框左、中、右（Dashboard 按 Q、W、E 選）。</t>
+          <t>- 若插入其他欄位，新欄位一定要有名稱；它們不會被讀取。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>- 距離：鎖定目標時 Dashboard 顯示的相機距離（不是捲尺），0.5–15 m，最多 2 位小數。</t>
+          <t>- 洞口：Dashboard 的編號 1–9（1 左下、2 左中、3 左上 … 9 右上）；10、11、12 是最上面的加分框左、中、右（Dashboard 按 Q、W、E 選）。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>- 仰角：Dashboard 的仰角脈寬，500–2500 的整數。</t>
+          <t>- 距離：鎖定目標時 Dashboard 顯示的相機距離（不是捲尺），0.5–15 m，最多 2 位小數。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- 轉速單位：用下拉選單選「%」或「us」，每一列可以不同。</t>
+          <t>- 仰角：Dashboard 的仰角脈寬，500–2500 的整數。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- 轉速：單位 % 時 0–100、最多 1 位小數；單位 us 時填 Dashboard「Falcon PWM」的脈寬整數，必須在正轉那一側（依 TuningConstants 的 Flywheel::INVERTED：false 是 1500–2000、true 是 1000–1500；產生這份 Excel 時是 1500–2000），會自動換算成 %。</t>
+          <t>- 轉速單位：用下拉選單選「%」或「us」，每一列可以不同。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- 列的順序不重要；空白列會略過；同一個洞口的同一個距離不能重複。</t>
+          <t>- 轉速：單位 % 時 0–100、最多 1 位小數；單位 us 時填 Dashboard「Falcon PWM」的脈寬整數，必須在正轉那一側（依 TuningConstants 的 Flywheel::INVERTED：false 是 1500–2000、true 是 1000–1500；產生這份 Excel 時是 1500–2000），會自動換算成 %。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- 資料請放在第 2–500 列；每個洞口最多 60 個點會畫進曲線圖。</t>
+          <t>- 列的順序不重要；空白列會略過；同一個洞口的同一個距離不能重複。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>- 資料請放在第 2–500 列；每個洞口最多 60 個點會畫進曲線圖。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>- 任何一格不符合，就不會產生檔案、也不會燒錄，畫面會指出是哪一格。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>沒有資料的洞</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- 會借用同一排中間洞的值：1、7 用 4，2、8 用 5，3、9 用 6。加分框（10–12）不借用：沒有資料就不會對它發射。</t>
+          <t>沒有資料的洞</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>- Mega 在兩個量測點之間用直線內插；比最近的點還近就用最近的點；比最遠的點還遠就用最遠的點。</t>
+          <t>- 會借用同一排中間洞的值：1、7 用 4，2、8 用 5，3、9 用 6，加分框 10、12 用 11（W）。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>- 曲線圖上的轉速曲線是 Excel 的乘冪趨勢線（y = a·x^b，從原點出發），只是用來看資料合不合理、哪個點量歪了；Mega 不是照這條曲線打。</t>
+          <t>- 中間洞（4、5、6、11）自己沒有資料時，那一排自動模式都不會發射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>- Mega 在兩個量測點之間用直線內插；比最近的點還近就用最近的點；比最遠的點還遠就用最遠的點。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
+        <is>
+          <t>- 曲線圖上的轉速曲線是 Excel 的乘冪趨勢線（y = a·x^b，從原點出發），只是用來看資料合不合理、哪個點量歪了；Mega 不是照這條曲線打。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>「圖表資料」是隱藏的工作表，由公式自動整理給曲線圖用，不用動它。</t>
         </is>

</xml_diff>

<commit_message>
Shot table: W (hole 11) 4.55 m / 65% / 1784 us from the 22:04 log (Jeremy's --import, re-run here; Q / E borrow it); tests no longer assume the bonus row is empty
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/shot_table/shot_table.xlsx
+++ b/tools/shot_table/shot_table.xlsx
@@ -1350,6 +1350,25 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26">
+        <v>11</v>
+      </c>
+      <c r="B26">
+        <v>4.55</v>
+      </c>
+      <c r="C26">
+        <v>1784</v>
+      </c>
+      <c r="D26">
+        <v>65</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="洞口" error="洞口要是 1–12 的整數（10–12 是加分框左中右）" sqref="A2:A500">

</xml_diff>